<commit_message>
Align Halcyon plan to InfinityStacks' requested AWS services
Record the infra request as submitted, and rework the design to use only Bedrock, IAM, S3, ECR,
Secrets Manager, RDS PostgreSQL, CloudWatch, Amplify and EC2: backend on EC2 with Docker Compose
and Caddy TLS, frontend on Amplify, a worker container instead of Lambda/EventBridge, AWS CLI
scripts instead of CDK. Day plan, security, risks and repo layout updated to match.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018mJx5VLNFyHg3anBqqcAy7
</commit_message>
<xml_diff>
--- a/hackathon/work/01-infra-request.xlsx
+++ b/hackathon/work/01-infra-request.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Infra Request" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Infra Request (submitted)" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -435,18 +435,18 @@
     <col width="18" customWidth="1" min="2" max="2"/>
     <col width="18" customWidth="1" min="3" max="3"/>
     <col width="18" customWidth="1" min="4" max="4"/>
-    <col width="48" customWidth="1" min="5" max="5"/>
-    <col width="48" customWidth="1" min="6" max="6"/>
-    <col width="48" customWidth="1" min="7" max="7"/>
-    <col width="48" customWidth="1" min="8" max="8"/>
-    <col width="48" customWidth="1" min="9" max="9"/>
-    <col width="48" customWidth="1" min="10" max="10"/>
-    <col width="48" customWidth="1" min="11" max="11"/>
-    <col width="48" customWidth="1" min="12" max="12"/>
-    <col width="48" customWidth="1" min="13" max="13"/>
-    <col width="48" customWidth="1" min="14" max="14"/>
-    <col width="48" customWidth="1" min="15" max="15"/>
-    <col width="48" customWidth="1" min="16" max="16"/>
+    <col width="40" customWidth="1" min="5" max="5"/>
+    <col width="40" customWidth="1" min="6" max="6"/>
+    <col width="40" customWidth="1" min="7" max="7"/>
+    <col width="40" customWidth="1" min="8" max="8"/>
+    <col width="40" customWidth="1" min="9" max="9"/>
+    <col width="40" customWidth="1" min="10" max="10"/>
+    <col width="40" customWidth="1" min="11" max="11"/>
+    <col width="40" customWidth="1" min="12" max="12"/>
+    <col width="40" customWidth="1" min="13" max="13"/>
+    <col width="40" customWidth="1" min="14" max="14"/>
+    <col width="40" customWidth="1" min="15" max="15"/>
+    <col width="40" customWidth="1" min="16" max="16"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -534,359 +534,180 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>[Team name]</t>
+          <t>InfinityStacks</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>[EMP ID]</t>
+          <t>7549</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>[Name]</t>
+          <t>Sravan Kumar D</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>smuthiki@evoketechnologies.com</t>
+          <t>sdayyala@evoketechnologies.com</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>• Backend: Python 3.11+ / FastAPI
-• Frontend: React + TypeScript (Next.js or Vite)
-• DB: PostgreSQL + DuckDB (analytics)
-• Docker</t>
-        </is>
-      </c>
-      <c r="F2" s="2" t="inlineStr">
-        <is>
-          <t>• pandas/polars, DuckDB, SQLAlchemy, Pydantic
-• scikit-learn, statsmodels, SimPy (what-if simulation)
-• Tailwind, shadcn/ui, Recharts/ECharts
-• pytest, Playwright
-• Anthropic SDK (Bedrock client) / Claude Agent SDK or LangGraph (agents)
-• Faker (synthetic data)</t>
-        </is>
-      </c>
+          <t>ReactJS, Python and AWS</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr"/>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>• Amazon Bedrock Runtime API with Anthropic Claude models (Sonnet-class agents, Haiku-class bulk extraction)
-• AWS SDK for Python (boto3): Bedrock, S3, Secrets Manager
-• No paid 3rd-party logistics APIs</t>
+          <t>Amazon Bedrock Runtime API</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>• Yes: 1 private repo for the team
-• Please confirm the official submission repo: the guidelines PDF says GitHub (we can mirror; CI/CD deploys to AWS)</t>
+          <t>GitHub.</t>
         </is>
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>• Claude Code (Evoke Claude) for all 3, with a raised usage limit / API credits beyond the 5-hour window
-• Cursor
-• GitHub Copilot</t>
+          <t>Claude Chat + Code</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>• AWS: 1 sandbox account (or an IAM role) for the hackathon period
-• Region ap-south-1 (Mumbai) with Bedrock cross-region inference; us-east-1 if Claude isn't enabled there</t>
+          <t>AWS</t>
         </is>
       </c>
       <c r="K2" s="2" t="inlineStr">
         <is>
-          <t>• Amazon Bedrock: Claude model access (Sonnet + Haiku). This is the AI service
-• ECS Fargate + ALB, or App Runner (API)
-• Amplify Hosting or S3 + CloudFront (frontend)
-• RDS PostgreSQL (db.t4g.micro/small, single-AZ)
-• S3 (data files, reports)
-• ECR
-• Secrets Manager
-• CloudWatch (logs/metrics, AI usage logs)
-• IAM deploy role + task roles with bedrock:InvokeModel
-• EC2 t3.large dev box only for members on CSC laptops</t>
-        </is>
-      </c>
-      <c r="L2" s="2" t="inlineStr">
-        <is>
-          <t>• None outside AWS: Claude via Amazon Bedrock
-• Carrier/EDI/WMS feeds simulated from the provided dataset</t>
-        </is>
-      </c>
-      <c r="M2" s="2" t="inlineStr">
-        <is>
-          <t>• Only the organiser-provided Problem 2 dataset (48,340 deliveries, WMS, EDI/API feeds, carrier events, complaint inbox, carrier preference sheet)
-• Synthetic data for gaps; no real personal/customer data</t>
-        </is>
-      </c>
-      <c r="N2" s="2" t="inlineStr">
-        <is>
-          <t>• Git, VS Code, Python 3.11+, Node.js 20 LTS, Docker Desktop, AWS CLI v2
-• Claude Code CLI, Cursor, GitHub Copilot extension
-• DBeaver/psql, Playwright browsers</t>
-        </is>
-      </c>
-      <c r="O2" s="2" t="inlineStr">
-        <is>
-          <t>• pypi.org, files.pythonhosted.org, registry.npmjs.org
-• github.com, *.githubusercontent.com, dev.azure.com
-• *.amazonaws.com (bedrock-runtime, ecr, s3), *.signin.aws.amazon.com, *.awsapps.com
-• *.amplifyapp.com, *.cloudfront.net, *.awsapprunner.com
-• api.anthropic.com, claude.ai (Claude Code)
-• playwright.azureedge.net, mcp.context7.com (optional)</t>
-        </is>
-      </c>
-      <c r="P2" s="2" t="inlineStr">
-        <is>
-          <t>• Full Problem 2 dataset + data dictionary (incl. how 'on-time' is computed)
-• Reachable URL for the deployed app (L1 check)
-• IAM/OIDC credentials for CI/CD deploys to AWS
-• AWS budget alert
-• Confirm agent logs in repo satisfy the 'AI usage logs' deliverable
-• Keep access until the L2 presentations (Nov week 1)</t>
-        </is>
-      </c>
+          <t>Amazon Bedrock (Claude AI model access), AWS IAM, Amazon S3 for document storage, AWS ECR, AWS Secrets Manager, PostgreSQL (Amazon RDS), CloudWatch for monitoring  AWS Amplify for frontend hosting, AWS EC2</t>
+        </is>
+      </c>
+      <c r="L2" s="2" t="inlineStr"/>
+      <c r="M2" s="2" t="inlineStr"/>
+      <c r="N2" s="2" t="inlineStr"/>
+      <c r="O2" s="2" t="inlineStr"/>
+      <c r="P2" s="2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>[Team name]</t>
+          <t>InfinityStacks</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>[EMP ID]</t>
+          <t>8388</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>[Name]</t>
+          <t>Sai M</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>[email]</t>
+          <t>smuthiki@evoketechnologies.com</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>• Backend: Python 3.11+ / FastAPI
-• Frontend: React + TypeScript (Next.js or Vite)
-• DB: PostgreSQL + DuckDB (analytics)
-• Docker</t>
+          <t>ReactJS, Python and AWS</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>• pandas/polars, DuckDB, SQLAlchemy, Pydantic
-• scikit-learn, statsmodels, SimPy (what-if simulation)
-• Tailwind, shadcn/ui, Recharts/ECharts
-• pytest, Playwright
-• Anthropic SDK (Bedrock client) / Claude Agent SDK or LangGraph (agents)
-• Faker (synthetic data)</t>
+          <t>Docker, Postman</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>• Amazon Bedrock Runtime API with Anthropic Claude models (Sonnet-class agents, Haiku-class bulk extraction)
-• AWS SDK for Python (boto3): Bedrock, S3, Secrets Manager
-• No paid 3rd-party logistics APIs</t>
+          <t>Amazon Bedrock Runtime API</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>• Yes: 1 private repo for the team
-• Please confirm the official submission repo: the guidelines PDF says GitHub (we can mirror; CI/CD deploys to AWS)</t>
+          <t>GitHub.</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>• Claude Code (Evoke Claude) for all 3, with a raised usage limit / API credits beyond the 5-hour window
-• Cursor
-• GitHub Copilot</t>
+          <t>Claude Chat + Code</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>• AWS: 1 sandbox account (or an IAM role) for the hackathon period
-• Region ap-south-1 (Mumbai) with Bedrock cross-region inference; us-east-1 if Claude isn't enabled there</t>
+          <t>AWS</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>• Amazon Bedrock: Claude model access (Sonnet + Haiku). This is the AI service
-• ECS Fargate + ALB, or App Runner (API)
-• Amplify Hosting or S3 + CloudFront (frontend)
-• RDS PostgreSQL (db.t4g.micro/small, single-AZ)
-• S3 (data files, reports)
-• ECR
-• Secrets Manager
-• CloudWatch (logs/metrics, AI usage logs)
-• IAM deploy role + task roles with bedrock:InvokeModel
-• EC2 t3.large dev box only for members on CSC laptops</t>
-        </is>
-      </c>
-      <c r="L3" s="2" t="inlineStr">
-        <is>
-          <t>• None outside AWS: Claude via Amazon Bedrock
-• Carrier/EDI/WMS feeds simulated from the provided dataset</t>
-        </is>
-      </c>
-      <c r="M3" s="2" t="inlineStr">
-        <is>
-          <t>• Only the organiser-provided Problem 2 dataset (48,340 deliveries, WMS, EDI/API feeds, carrier events, complaint inbox, carrier preference sheet)
-• Synthetic data for gaps; no real personal/customer data</t>
-        </is>
-      </c>
-      <c r="N3" s="2" t="inlineStr">
-        <is>
-          <t>• Git, VS Code, Python 3.11+, Node.js 20 LTS, Docker Desktop, AWS CLI v2
-• Claude Code CLI, Cursor, GitHub Copilot extension
-• DBeaver/psql, Playwright browsers</t>
-        </is>
-      </c>
-      <c r="O3" s="2" t="inlineStr">
-        <is>
-          <t>• pypi.org, files.pythonhosted.org, registry.npmjs.org
-• github.com, *.githubusercontent.com, dev.azure.com
-• *.amazonaws.com (bedrock-runtime, ecr, s3), *.signin.aws.amazon.com, *.awsapps.com
-• *.amplifyapp.com, *.cloudfront.net, *.awsapprunner.com
-• api.anthropic.com, claude.ai (Claude Code)
-• playwright.azureedge.net, mcp.context7.com (optional)</t>
-        </is>
-      </c>
-      <c r="P3" s="2" t="inlineStr">
-        <is>
-          <t>• Full Problem 2 dataset + data dictionary (incl. how 'on-time' is computed)
-• Reachable URL for the deployed app (L1 check)
-• IAM/OIDC credentials for CI/CD deploys to AWS
-• AWS budget alert
-• Confirm agent logs in repo satisfy the 'AI usage logs' deliverable
-• Keep access until the L2 presentations (Nov week 1)</t>
-        </is>
-      </c>
+          <t>Amazon Bedrock (Claude AI model access), AWS IAM, Amazon S3 for document storage, AWS ECR, AWS Secrets Manager, PostgreSQL (Amazon RDS), CloudWatch for monitoring  AWS Amplify for frontend hosting, AWS EC2</t>
+        </is>
+      </c>
+      <c r="L3" s="2" t="inlineStr"/>
+      <c r="M3" s="2" t="inlineStr"/>
+      <c r="N3" s="2" t="inlineStr"/>
+      <c r="O3" s="2" t="inlineStr"/>
+      <c r="P3" s="2" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>[Team name]</t>
+          <t>InfinityStacks</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>[EMP ID]</t>
+          <t>5511</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>[Name]</t>
+          <t>Dinesh K</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>[email]</t>
+          <t>dkarasu@evoketechnologies.com</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>• Backend: Python 3.11+ / FastAPI
-• Frontend: React + TypeScript (Next.js or Vite)
-• DB: PostgreSQL + DuckDB (analytics)
-• Docker</t>
-        </is>
-      </c>
-      <c r="F4" s="2" t="inlineStr">
-        <is>
-          <t>• pandas/polars, DuckDB, SQLAlchemy, Pydantic
-• scikit-learn, statsmodels, SimPy (what-if simulation)
-• Tailwind, shadcn/ui, Recharts/ECharts
-• pytest, Playwright
-• Anthropic SDK (Bedrock client) / Claude Agent SDK or LangGraph (agents)
-• Faker (synthetic data)</t>
-        </is>
-      </c>
+          <t>ReactJS, Python and AWS</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr"/>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>• Amazon Bedrock Runtime API with Anthropic Claude models (Sonnet-class agents, Haiku-class bulk extraction)
-• AWS SDK for Python (boto3): Bedrock, S3, Secrets Manager
-• No paid 3rd-party logistics APIs</t>
+          <t>Amazon Bedrock Runtime API</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>• Yes: 1 private repo for the team
-• Please confirm the official submission repo: the guidelines PDF says GitHub (we can mirror; CI/CD deploys to AWS)</t>
+          <t>GitHub.</t>
         </is>
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>• Claude Code (Evoke Claude) for all 3, with a raised usage limit / API credits beyond the 5-hour window
-• Cursor
-• GitHub Copilot</t>
+          <t>Claude Chat + Code</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>• AWS: 1 sandbox account (or an IAM role) for the hackathon period
-• Region ap-south-1 (Mumbai) with Bedrock cross-region inference; us-east-1 if Claude isn't enabled there</t>
+          <t>AWS</t>
         </is>
       </c>
       <c r="K4" s="2" t="inlineStr">
         <is>
-          <t>• Amazon Bedrock: Claude model access (Sonnet + Haiku). This is the AI service
-• ECS Fargate + ALB, or App Runner (API)
-• Amplify Hosting or S3 + CloudFront (frontend)
-• RDS PostgreSQL (db.t4g.micro/small, single-AZ)
-• S3 (data files, reports)
-• ECR
-• Secrets Manager
-• CloudWatch (logs/metrics, AI usage logs)
-• IAM deploy role + task roles with bedrock:InvokeModel
-• EC2 t3.large dev box only for members on CSC laptops</t>
-        </is>
-      </c>
-      <c r="L4" s="2" t="inlineStr">
-        <is>
-          <t>• None outside AWS: Claude via Amazon Bedrock
-• Carrier/EDI/WMS feeds simulated from the provided dataset</t>
-        </is>
-      </c>
-      <c r="M4" s="2" t="inlineStr">
-        <is>
-          <t>• Only the organiser-provided Problem 2 dataset (48,340 deliveries, WMS, EDI/API feeds, carrier events, complaint inbox, carrier preference sheet)
-• Synthetic data for gaps; no real personal/customer data</t>
-        </is>
-      </c>
-      <c r="N4" s="2" t="inlineStr">
-        <is>
-          <t>• Git, VS Code, Python 3.11+, Node.js 20 LTS, Docker Desktop, AWS CLI v2
-• Claude Code CLI, Cursor, GitHub Copilot extension
-• DBeaver/psql, Playwright browsers</t>
-        </is>
-      </c>
-      <c r="O4" s="2" t="inlineStr">
-        <is>
-          <t>• pypi.org, files.pythonhosted.org, registry.npmjs.org
-• github.com, *.githubusercontent.com, dev.azure.com
-• *.amazonaws.com (bedrock-runtime, ecr, s3), *.signin.aws.amazon.com, *.awsapps.com
-• *.amplifyapp.com, *.cloudfront.net, *.awsapprunner.com
-• api.anthropic.com, claude.ai (Claude Code)
-• playwright.azureedge.net, mcp.context7.com (optional)</t>
-        </is>
-      </c>
-      <c r="P4" s="2" t="inlineStr">
-        <is>
-          <t>• Full Problem 2 dataset + data dictionary (incl. how 'on-time' is computed)
-• Reachable URL for the deployed app (L1 check)
-• IAM/OIDC credentials for CI/CD deploys to AWS
-• AWS budget alert
-• Confirm agent logs in repo satisfy the 'AI usage logs' deliverable
-• Keep access until the L2 presentations (Nov week 1)</t>
-        </is>
-      </c>
+          <t>Amazon Bedrock (Claude AI model access), AWS IAM, Amazon S3 for document storage, AWS ECR, AWS Secrets Manager, PostgreSQL (Amazon RDS), CloudWatch for monitoring  AWS Amplify for frontend hosting, AWS EC2</t>
+        </is>
+      </c>
+      <c r="L4" s="2" t="inlineStr"/>
+      <c r="M4" s="2" t="inlineStr"/>
+      <c r="N4" s="2" t="inlineStr"/>
+      <c r="O4" s="2" t="inlineStr"/>
+      <c r="P4" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>